<commit_message>
Updated Excel file 24-09
</commit_message>
<xml_diff>
--- a/12623794.xlsx
+++ b/12623794.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c77697d53e5dee5/Desktop/LPU/Python/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="471" documentId="13_ncr:1_{A8837051-77D3-4D36-92D2-5680DDD8E381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC3FE973-76A4-47C7-AE8D-EEF07859F455}"/>
+  <xr:revisionPtr revIDLastSave="483" documentId="13_ncr:1_{A8837051-77D3-4D36-92D2-5680DDD8E381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97EFE702-646E-4F1E-909A-86E035D880A8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="97">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -324,6 +324,9 @@
   <si>
     <t>Normalization in DBMS,in between like in DBMS</t>
   </si>
+  <si>
+    <t>Blood relation,static routers connection</t>
+  </si>
 </sst>
 </file>
 
@@ -606,6 +609,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2710,27 +2717,51 @@
         <v>95</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14"/>
-      <c r="D41" s="14"/>
-      <c r="E41" s="14"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="14"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="15" t="str">
+    <row r="41" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B41" s="14">
+        <v>450</v>
+      </c>
+      <c r="C41" s="14">
+        <v>40</v>
+      </c>
+      <c r="D41" s="14">
+        <v>80</v>
+      </c>
+      <c r="E41" s="14">
+        <v>40</v>
+      </c>
+      <c r="F41" s="14">
+        <v>6</v>
+      </c>
+      <c r="G41" s="14">
+        <v>350</v>
+      </c>
+      <c r="H41" s="14">
+        <v>120</v>
+      </c>
+      <c r="I41" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J41" s="15" t="str">
+        <v>736</v>
+      </c>
+      <c r="J41" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="16"/>
-      <c r="M41" s="16"/>
-      <c r="N41" s="17"/>
+        <v>704</v>
+      </c>
+      <c r="K41" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L41" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M41" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N41" s="17" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" s="13"/>
@@ -10747,6 +10778,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>